<commit_message>
Replaced "fragmentation" and "frag" with "density" and "dens" throughout, because I was confusing myself
</commit_message>
<xml_diff>
--- a/outputs/frag_stats_90m_RAN.xlsx
+++ b/outputs/frag_stats_90m_RAN.xlsx
@@ -1,6 +1,6 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" mc:Ignorable="x15 xr xr6 xr10">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24228"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
@@ -8,13 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\raenb\Documents\GitHub\madagascar\outputs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:40009_{2BEE99E6-5637-4128-B8AF-6B53E8ACE820}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C8EA610B-2FCE-4DE4-879D-A64705F645BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-1035" windowWidth="29040" windowHeight="15840" activeTab="1"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="frag_stats_90m" sheetId="1" r:id="rId1"/>
-    <sheet name="reorg" sheetId="2" r:id="rId2"/>
+    <sheet name="reorganized" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
@@ -74,7 +74,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="18" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -648,7 +648,7 @@
           <c:order val="0"/>
           <c:tx>
             <c:strRef>
-              <c:f>reorg!$B$1</c:f>
+              <c:f>reorganized!$B$1</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -673,7 +673,7 @@
             <c:noEndCap val="0"/>
             <c:plus>
               <c:numRef>
-                <c:f>reorg!$E$2:$E$4</c:f>
+                <c:f>reorganized!$E$2:$E$4</c:f>
                 <c:numCache>
                   <c:formatCode>General</c:formatCode>
                   <c:ptCount val="3"/>
@@ -691,7 +691,7 @@
             </c:plus>
             <c:minus>
               <c:numRef>
-                <c:f>reorg!$E$2:$E$4</c:f>
+                <c:f>reorganized!$E$2:$E$4</c:f>
                 <c:numCache>
                   <c:formatCode>General</c:formatCode>
                   <c:ptCount val="3"/>
@@ -720,7 +720,7 @@
           </c:errBars>
           <c:cat>
             <c:numRef>
-              <c:f>reorg!$A$2:$A$4</c:f>
+              <c:f>reorganized!$A$2:$A$4</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="3"/>
@@ -738,7 +738,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>reorg!$B$2:$B$4</c:f>
+              <c:f>reorganized!$B$2:$B$4</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="3"/>
@@ -765,7 +765,7 @@
           <c:order val="1"/>
           <c:tx>
             <c:strRef>
-              <c:f>reorg!$C$1</c:f>
+              <c:f>reorganized!$C$1</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -790,7 +790,7 @@
             <c:noEndCap val="0"/>
             <c:plus>
               <c:numRef>
-                <c:f>reorg!$F$2:$F$4</c:f>
+                <c:f>reorganized!$F$2:$F$4</c:f>
                 <c:numCache>
                   <c:formatCode>General</c:formatCode>
                   <c:ptCount val="3"/>
@@ -808,7 +808,7 @@
             </c:plus>
             <c:minus>
               <c:numRef>
-                <c:f>reorg!$F$2:$F$4</c:f>
+                <c:f>reorganized!$F$2:$F$4</c:f>
                 <c:numCache>
                   <c:formatCode>General</c:formatCode>
                   <c:ptCount val="3"/>
@@ -837,7 +837,7 @@
           </c:errBars>
           <c:val>
             <c:numRef>
-              <c:f>reorg!$C$2:$C$4</c:f>
+              <c:f>reorganized!$C$2:$C$4</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="3"/>
@@ -864,7 +864,7 @@
           <c:order val="2"/>
           <c:tx>
             <c:strRef>
-              <c:f>reorg!$D$1</c:f>
+              <c:f>reorganized!$D$1</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -889,7 +889,7 @@
             <c:noEndCap val="0"/>
             <c:plus>
               <c:numRef>
-                <c:f>reorg!$G$2:$G$4</c:f>
+                <c:f>reorganized!$G$2:$G$4</c:f>
                 <c:numCache>
                   <c:formatCode>General</c:formatCode>
                   <c:ptCount val="3"/>
@@ -907,7 +907,7 @@
             </c:plus>
             <c:minus>
               <c:numRef>
-                <c:f>reorg!$G$2:$G$4</c:f>
+                <c:f>reorganized!$G$2:$G$4</c:f>
                 <c:numCache>
                   <c:formatCode>General</c:formatCode>
                   <c:ptCount val="3"/>
@@ -936,7 +936,7 @@
           </c:errBars>
           <c:val>
             <c:numRef>
-              <c:f>reorg!$D$2:$D$4</c:f>
+              <c:f>reorganized!$D$2:$D$4</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="3"/>
@@ -1225,7 +1225,7 @@
           <c:order val="0"/>
           <c:tx>
             <c:strRef>
-              <c:f>reorg!$B$1</c:f>
+              <c:f>reorganized!$B$1</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -1265,7 +1265,7 @@
             <c:noEndCap val="0"/>
             <c:plus>
               <c:numRef>
-                <c:f>reorg!$E$2:$E$4</c:f>
+                <c:f>reorganized!$E$2:$E$4</c:f>
                 <c:numCache>
                   <c:formatCode>General</c:formatCode>
                   <c:ptCount val="3"/>
@@ -1283,7 +1283,7 @@
             </c:plus>
             <c:minus>
               <c:numRef>
-                <c:f>reorg!$E$2:$E$4</c:f>
+                <c:f>reorganized!$E$2:$E$4</c:f>
                 <c:numCache>
                   <c:formatCode>General</c:formatCode>
                   <c:ptCount val="3"/>
@@ -1312,7 +1312,7 @@
           </c:errBars>
           <c:cat>
             <c:numRef>
-              <c:f>reorg!$A$2:$A$4</c:f>
+              <c:f>reorganized!$A$2:$A$4</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="3"/>
@@ -1330,7 +1330,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>reorg!$B$2:$B$4</c:f>
+              <c:f>reorganized!$B$2:$B$4</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="3"/>
@@ -1621,7 +1621,7 @@
           <c:order val="0"/>
           <c:tx>
             <c:strRef>
-              <c:f>reorg!$D$1</c:f>
+              <c:f>reorganized!$D$1</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -1661,7 +1661,7 @@
             <c:noEndCap val="0"/>
             <c:plus>
               <c:numRef>
-                <c:f>reorg!$G$2:$G$4</c:f>
+                <c:f>reorganized!$G$2:$G$4</c:f>
                 <c:numCache>
                   <c:formatCode>General</c:formatCode>
                   <c:ptCount val="3"/>
@@ -1679,7 +1679,7 @@
             </c:plus>
             <c:minus>
               <c:numRef>
-                <c:f>reorg!$G$2:$G$4</c:f>
+                <c:f>reorganized!$G$2:$G$4</c:f>
                 <c:numCache>
                   <c:formatCode>General</c:formatCode>
                   <c:ptCount val="3"/>
@@ -1710,7 +1710,7 @@
           </c:errBars>
           <c:val>
             <c:numRef>
-              <c:f>reorg!$D$2:$D$4</c:f>
+              <c:f>reorganized!$D$2:$D$4</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="3"/>
@@ -2001,7 +2001,7 @@
           <c:order val="0"/>
           <c:tx>
             <c:strRef>
-              <c:f>reorg!$C$1</c:f>
+              <c:f>reorganized!$C$1</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -2041,7 +2041,7 @@
             <c:noEndCap val="0"/>
             <c:plus>
               <c:numRef>
-                <c:f>reorg!$F$2:$F$4</c:f>
+                <c:f>reorganized!$F$2:$F$4</c:f>
                 <c:numCache>
                   <c:formatCode>General</c:formatCode>
                   <c:ptCount val="3"/>
@@ -2059,7 +2059,7 @@
             </c:plus>
             <c:minus>
               <c:numRef>
-                <c:f>reorg!$F$2:$F$4</c:f>
+                <c:f>reorganized!$F$2:$F$4</c:f>
                 <c:numCache>
                   <c:formatCode>General</c:formatCode>
                   <c:ptCount val="3"/>
@@ -2088,7 +2088,7 @@
           </c:errBars>
           <c:val>
             <c:numRef>
-              <c:f>reorg!$C$2:$C$4</c:f>
+              <c:f>reorganized!$C$2:$C$4</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="3"/>
@@ -4989,7 +4989,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:G5"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -5119,7 +5119,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:G4"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>

</xml_diff>